<commit_message>
Add graded optional hints to EGO quizzes
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R590d369223504e40"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Ra4479cc3498c4be5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rbb378f87db8c41f4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R144d727c1aa84af1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3405,6 +3405,28 @@
         <x:v>EGO와 EGO 기프트 결과 화면에서 정답 정보와 이미지가 추측 기록보다 먼저 보이도록 상단으로 옮겼습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="131" ht="86.4000015258789" hidden="0" customHeight="1">
+      <x:c r="A131" t="str">
+        <x:v>v0.16.0</x:v>
+      </x:c>
+      <x:c r="B131" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C131" t="str">
+        <x:v>EGO와 EGO 기프트 퀴즈에 필요한 정보만 고르는 선택형 힌트 패널 추가.
+추측 1회와 유료 힌트 1개를 각각 비용 1로 합산하고, 정답 시 비용 1~2 ALEPH·3~4 WAW·5~6 HE·7~8 TETH·9 이상 ZAYIN 관리자 평가 적용.
+EGO와 EGO 기프트의 힌트·비용 상태를 독립 저장해 일일 진행 복원과 결과·공유 카드에 반영.
+EGO 기프트는 첫 효과 기록을 무료로 제공하고 이후 효과 기록을 수동 공개하도록 변경. 등급·조건 속성·이름 길이·강화 가능·키워드도 개별 공개 가능.
+전용 테마 팩 정보를 효과 기록 단서에 포함하고 기프트 데이터 441개 재빌드.
+브라우저에서 선택 힌트 비용, 오답 추측 비용, 효과 기록 수동 공개, 키워드 가림 해제와 콘솔 오류 없음 확인.</x:v>
+      </x:c>
+      <x:c r="D131" t="str">
+        <x:v>EGO와 EGO 기프트 퀴즈에 원하는 힌트만 골라 보는 기능을 추가했습니다. 추측과 유료 힌트는 각각 비용 1이며, 비용이 적을수록 ALEPH에 가까운 높은 관리자 평가를 받습니다.
+EGO와 기프트의 비용은 서로 섞이지 않습니다. 기프트의 첫 효과 기록은 무료이며, 다음 효과 기록과 등급·조건 속성·이름 길이·강화 가능·키워드를 필요한 만큼 직접 열 수 있습니다.</x:v>
+      </x:c>
+      <x:c r="E131"/>
+      <x:c r="F131"/>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Refine EGO hints and home status
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rbb378f87db8c41f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R144d727c1aa84af1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rcf7c83718efb4565"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rfb57ed8535ad44ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3427,6 +3427,39 @@
       <x:c r="E131"/>
       <x:c r="F131"/>
     </x:row>
+    <x:row r="132">
+      <x:c r="A132" t="str">
+        <x:v>v0.16.1</x:v>
+      </x:c>
+      <x:c r="B132" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C132" t="str">
+        <x:v>홈 화면에 최신 반영 인격 상태 표시를 추가함. identityUpdates.json의 마지막 identity 항목을 data.json과 연결해 인격명과 ID를 표시하고, 전체 인격 수도 함께 갱신함. 비동기 로드 순서와 업데이트 목록 누락 시 폴백 문구를 처리함.</x:v>
+      </x:c>
+      <x:c r="D132" t="str">
+        <x:v>홈 화면에서 사이트에 마지막으로 반영된 인격의 이름과 ID, 전체 인격 수를 확인할 수 있습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="133" ht="57.599998474121094" hidden="0" customHeight="1">
+      <x:c r="A133" t="str">
+        <x:v>v0.16.2</x:v>
+      </x:c>
+      <x:c r="B133" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C133" t="str">
+        <x:v>EGO 자원 구성 힌트를 클릭마다 자원 1개씩 공개하도록 변경하고, 각 자원 공개를 힌트 비용 1로 독립 합산함. 일일 상태와 결과 기록에 resourceRevealCount를 저장하며 구버전 저장 상태도 호환 처리함.
+공개된 힌트 버튼의 disabled opacity를 해제하고 대비·배경·테두리를 강화해 열린 정보를 선명하게 표시함.
+EGO 기프트 효과 기록의 기본 무료 공개를 제거하고 0개 공개 상태에서 시작하도록 변경함. 첫 효과 기록부터 공개할 때마다 비용 1을 부과함.
+검증: EGO 자원 0/5→1/5 비용 1→2/5 비용 2, 기프트 효과 0/2→1/2 비용 1, ALEPH/WAW 예상 등급 전환과 브라우저 콘솔 오류 없음을 확인함.</x:v>
+      </x:c>
+      <x:c r="D133" t="str">
+        <x:v>EGO 자원 구성은 누를 때마다 자원 하나씩 공개되며, 각각 힌트 비용 1로 계산됩니다.
+열어 본 힌트는 흐려지지 않고 선명하게 표시됩니다.
+EGO 기프트 효과 기록은 처음부터 보이지 않으며 첫 기록부터 비용 1을 내고 열어야 합니다. 따라서 ALEPH는 힌트를 최대 1개만 열고 첫 추측에 맞힌 경우까지 받을 수 있습니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Move-in Registration Heathcliff EGO
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rcf7c83718efb4565"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rfb57ed8535ad44ee"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R454e4b8b5d5a4472"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rb02321093241439e"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3460,6 +3460,20 @@
 EGO 기프트 효과 기록은 처음부터 보이지 않으며 첫 기록부터 비용 1을 내고 열어야 합니다. 따라서 ALEPH는 힌트를 최대 1개만 열고 첫 추측에 맞힌 경우까지 받을 수 있습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="134">
+      <x:c r="A134" t="str">
+        <x:v>v0.16.3</x:v>
+      </x:c>
+      <x:c r="B134" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C134" t="str">
+        <x:v>기존 EGOData의 '입주 신고' 히스클리프(ID 119) 행을 유지하고 아이콘 경로를 신규 원본 PNG(./images/ego/119.png)로 교체함. build-content-updates.js에 latestIdentityId를 별도 보존해 신규 EGO만 감지된 빌드에서도 홈의 최신 인격 표시가 유지되도록 수정. 신규 콘텐츠 안내는 EGO 119만 최초 1회 표시되도록 검증.</x:v>
+      </x:c>
+      <x:c r="D134" t="str">
+        <x:v>히스클리프 EGO '입주 신고'의 원본 이미지를 추가했습니다. 새로 접속하면 신규 EGO 안내에서 한 번 확인할 수 있습니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Show latest EGO on home
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R454e4b8b5d5a4472"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rb02321093241439e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R3700b3330e5a4c84"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Re3a6d97caf8c44b2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3474,6 +3474,20 @@
         <x:v>히스클리프 EGO '입주 신고'의 원본 이미지를 추가했습니다. 새로 접속하면 신규 EGO 안내에서 한 번 확인할 수 있습니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="135">
+      <x:c r="A135" t="str">
+        <x:v>v0.16.4</x:v>
+      </x:c>
+      <x:c r="B135" t="str">
+        <x:v>2026-09-17</x:v>
+      </x:c>
+      <x:c r="C135" t="str">
+        <x:v>홈의 최신 반영 상태를 인격과 EGO 두 행으로 확장함. identityUpdates.json에 latestEgoId를 별도 저장하고, 신규 인격 또는 EGO만 추가된 빌드에서도 두 최신 항목을 각각 유지하도록 build-content-updates.js를 수정함. EGO 데이터 로드 완료 시 이름, 수감자, 등급, ID, 전체 EGO 수를 갱신하도록 처리함.</x:v>
+      </x:c>
+      <x:c r="D135" t="str">
+        <x:v>홈 화면에서 마지막으로 반영된 인격과 EGO를 함께 확인할 수 있습니다. EGO만 업데이트된 경우에도 최신 EGO 이름, 수감자, 등급, ID가 표시됩니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Add Haute Couture Rodion and two EGO updates
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R3700b3330e5a4c84"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Re3a6d97caf8c44b2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R9a9b76d4488c4664"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="R4d9565e1cbcc44c1"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3488,6 +3488,37 @@
         <x:v>홈 화면에서 마지막으로 반영된 인격과 EGO를 함께 확인할 수 있습니다. EGO만 업데이트된 경우에도 최신 EGO 이름, 수감자, 등급, ID가 표시됩니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="136">
+      <x:c r="A136" t="str">
+        <x:v>v0.16.5</x:v>
+      </x:c>
+      <x:c r="B136" t="str">
+        <x:v>2026-09-22</x:v>
+      </x:c>
+      <x:c r="C136" t="str">
+        <x:v>홈 최신 반영 상태에서 내부 ID 문구를 제거함. 인격·EGO 행을 각각 키보드 접근 가능한 버튼으로 바꾸고, 선택한 종류의 최신 추가 카드만 신규 콘텐츠 팝업에 표시하도록 연결함.</x:v>
+      </x:c>
+      <x:c r="D136" t="str">
+        <x:v>홈의 최신 반영 인격과 EGO에서 ID 표기를 제거했습니다.
+최신 인격과 최신 EGO를 각각 누르면 해당 종류의 추가 소식을 따로 확인할 수 있습니다.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="137">
+      <x:c r="A137" t="str">
+        <x:v>v0.16.6</x:v>
+      </x:c>
+      <x:c r="B137" t="str">
+        <x:v>2026-10-01</x:v>
+      </x:c>
+      <x:c r="C137" t="str">
+        <x:v>신규 인격 오트쿠튀르::수선실 로쟈(ID 10917)와 신규 EGO 거울촉각 로쟈(ID 128), 거절선포 홍루(ID 129)의 데이터·WebP 이미지를 추가함. identityUpdates.json에 latestIdentityIds/latestEgoIds 배열을 도입해 동일 빌드에서 같은 종류가 여러 개 추가돼도 홈 상태와 종류별 팝업이 전부 표시하도록 확장하고 기존 단일 ID 필드 폴백을 유지함.</x:v>
+      </x:c>
+      <x:c r="D137" t="str">
+        <x:v>신규 인격 '오트쿠튀르::수선실 로쟈'를 추가했습니다.
+신규 EGO '거울촉각 로쟈'와 '거절선포 홍루'를 추가했습니다.
+같은 업데이트에 인격이나 EGO가 여러 개 추가되면 홈 최신 반영 상태와 팝업에 모두 표시됩니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>

<commit_message>
Release v0.16.8 with enkephalin activity and visual quizzes
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -325,7 +325,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F138"/>
+  <dimension ref="A1:F139"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3654,6 +3654,33 @@
 TRY 기록의 항목별 일치 판정과 방향 표시를 없애고, 제출한 EGO·기프트의 큰 이미지와 정보를 표시합니다. EGO 이미지는 원형으로 통일했으며 정답 TRY는 초록색으로 강조합니다.
 상단에 도움말과 포기 버튼을 모으고 안내 문구를 정리했습니다. 결과에는 전체 등급 기준과 내 등급이 표시됩니다.
 죄악 아이콘을 개선하고, 빌드 후 index.html 파일을 직접 열어도 퀴즈 데이터를 불러올 수 있도록 수정했습니다.</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>v0.16.8</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>2026-10-01</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>이미지 퀴즈 데이터·빌드·검증 스크립트 및 로컬 WebP 자산 추가.
+일일 엔케팔린 기록·등급 산정·과거 기록 재계산·활동 그래프·지령 카드 회수 미터 구현.
+ZAYIN/TETH/HE/WAW/ALEPH 등급 WebP 자산과 EGO·기프트 결과 평가 표식 통합.</t>
+        </is>
+      </c>
+      <c r="D139" t="inlineStr">
+        <is>
+          <t>관리자 식별 교육에 인물·보스·패닉 이미지 퀴즈를 추가했습니다.
+오늘의 인격·EGO·EGO 기프트에 엔케팔린 배정량과 회수량을 적용하고, 획득량에 따라 ZAYIN부터 ALEPH까지 등급을 표시합니다.
+홈에 최근 7일 엔케팔린 획득량과 일별 종합 등급을 보여주는 액체 막대 그래프를 추가했습니다.
+오늘의 지령 카드에서 등급 이미지, 획득 엔케팔린, 배정량 대비 회수 바를 함께 확인할 수 있습니다.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Refine EGO result summaries
</commit_message>
<xml_diff>
--- a/UpdateLog.xlsx
+++ b/UpdateLog.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="R3b3ed0bc462a45e5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Ra916c258ab7d442f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog" sheetId="1" r:id="Rd9d5960b308f4866"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="UpdateLog_백업" sheetId="2" r:id="Rb97344e3db2f4674"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -3695,6 +3695,20 @@
 TRY 번호는 실제 제출 순서대로 유지됩니다.</x:v>
       </x:c>
     </x:row>
+    <x:row r="141">
+      <x:c r="A141" t="str">
+        <x:v>v0.16.10</x:v>
+      </x:c>
+      <x:c r="B141" t="str">
+        <x:v>2026-10-01</x:v>
+      </x:c>
+      <x:c r="C141" t="str">
+        <x:v>오늘의 EGO와 EGO 기프트 결과 화면에서 정답 이미지를 관리자 등급 영역 바로 아래로 이동. 엔케팔린 회수 결과와 전체 등급 기준표를 하나의 통합 카드로 묶고, 상세 정보와 효과는 이미지 아래에 배치. 두 결과 렌더러의 순서를 검증하는 회귀 테스트 추가.</x:v>
+      </x:c>
+      <x:c r="D141" t="str">
+        <x:v>오늘의 EGO와 EGO 기프트 결과에서 엔케팔린 회수 등급과 등급 기준표가 하나의 카드로 표시됩니다. 그 아래에 정답 이미지가 크게 나오고, 상세 정보와 효과가 이어집니다.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>

</xml_diff>